<commit_message>
edits following user review. still need to resolve the folder re-oreg
</commit_message>
<xml_diff>
--- a/dist/files/sample_project/soil samples.xlsx
+++ b/dist/files/sample_project/soil samples.xlsx
@@ -498,8 +498,8 @@
       <c r="B5">
         <v>15.1</v>
       </c>
-      <c r="C5">
-        <v>42.1</v>
+      <c r="C5" t="str">
+        <v>42,1</v>
       </c>
       <c r="D5">
         <v>4.1</v>

</xml_diff>